<commit_message>
Quickstart logic and docs improvement | Ensure imported ODCS brings the transformLogic with | Bring transformLogic into DBT code
</commit_message>
<xml_diff>
--- a/python/src/dbt_data_engineering_toolkit_compiler/resources/data_product.xlsx
+++ b/python/src/dbt_data_engineering_toolkit_compiler/resources/data_product.xlsx
@@ -1,35 +1,35 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <sheets>
-    <sheet name="Instructions" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="Fundamentals" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="Schema data_product" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet name="Relationships" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet name="Quality" sheetId="5" state="visible" r:id="rId5"/>
-    <sheet name="Support" sheetId="6" state="visible" r:id="rId6"/>
-    <sheet name="Team" sheetId="7" state="visible" r:id="rId7"/>
-    <sheet name="Roles" sheetId="8" state="visible" r:id="rId8"/>
-    <sheet name="SLA" sheetId="9" state="visible" r:id="rId9"/>
-    <sheet name="Servers" sheetId="10" state="visible" r:id="rId10"/>
-    <sheet name="Pricing" sheetId="11" state="visible" r:id="rId11"/>
-    <sheet name="Custom Properties" sheetId="12" state="visible" r:id="rId12"/>
-    <sheet name="DET Models" sheetId="13" state="visible" r:id="rId13"/>
-    <sheet name="DET Model Inputs" sheetId="14" state="visible" r:id="rId14"/>
-    <sheet name="DET Sources" sheetId="15" state="visible" r:id="rId15"/>
-    <sheet name="DET Source Schema" sheetId="16" state="visible" r:id="rId16"/>
-    <sheet name="DET Mapping" sheetId="17" state="visible" r:id="rId17"/>
-    <sheet name="DET Parameters" sheetId="18" state="visible" r:id="rId18"/>
-    <sheet name="DET Relationships" sheetId="19" state="visible" r:id="rId19"/>
-    <sheet name="Operational Validation" sheetId="20" state="visible" r:id="rId20"/>
-    <sheet name="Operational Parameters" sheetId="21" state="visible" r:id="rId21"/>
-    <sheet name="DET Lookups" sheetId="22" state="visible" r:id="rId22"/>
-    <sheet name="DET Build" sheetId="23" state="visible" r:id="rId23"/>
-    <sheet name="_DET Lists" sheetId="24" state="veryHidden" r:id="rId24"/>
-    <sheet name="_DET Metadata" sheetId="25" state="veryHidden" r:id="rId25"/>
-    <sheet name="_DET Context" sheetId="26" state="veryHidden" r:id="rId26"/>
-    <sheet name="_DET Raw ODCS" sheetId="27" state="veryHidden" r:id="rId27"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Instructions" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Fundamentals" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Schema data_product" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Relationships" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Quality" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Support" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Team" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Roles" sheetId="8" state="visible" r:id="rId8"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SLA" sheetId="9" state="visible" r:id="rId9"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Servers" sheetId="10" state="visible" r:id="rId10"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Pricing" sheetId="11" state="visible" r:id="rId11"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Custom Properties" sheetId="12" state="visible" r:id="rId12"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="DET Models" sheetId="13" state="visible" r:id="rId13"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="DET Model Inputs" sheetId="14" state="visible" r:id="rId14"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="DET Sources" sheetId="15" state="visible" r:id="rId15"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="DET Source Schema" sheetId="16" state="visible" r:id="rId16"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="DET Mapping" sheetId="17" state="visible" r:id="rId17"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="DET Parameters" sheetId="18" state="visible" r:id="rId18"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="DET Relationships" sheetId="19" state="visible" r:id="rId19"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Operational Validation" sheetId="20" state="visible" r:id="rId20"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Operational Parameters" sheetId="21" state="visible" r:id="rId21"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="DET Lookups" sheetId="22" state="visible" r:id="rId22"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="DET Build" sheetId="23" state="visible" r:id="rId23"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="_DET Lists" sheetId="24" state="veryHidden" r:id="rId24"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="_DET Metadata" sheetId="25" state="veryHidden" r:id="rId25"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="_DET Context" sheetId="26" state="veryHidden" r:id="rId26"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="_DET Raw ODCS" sheetId="27" state="veryHidden" r:id="rId27"/>
   </sheets>
   <definedNames>
     <definedName name="apiVersion">Fundamentals!$C$5</definedName>
@@ -126,30 +126,32 @@
     <definedName name="_DET_OP_clean_phone">'_DET Context'!$I$2:$I$2</definedName>
     <definedName name="_DET_OP_clean_text">'_DET Context'!$J$2:$J$5</definedName>
     <definedName name="_DET_OP_clean_timestamp">'_DET Context'!$K$2:$K$2</definedName>
-    <definedName name="_DET_OP_copy">'_DET Context'!$L$2:$L$2</definedName>
-    <definedName name="_DET_OP_correct_errors">'_DET Context'!$M$2:$M$3</definedName>
-    <definedName name="_DET_OP_fill_missing">'_DET Context'!$N$2:$N$2</definedName>
-    <definedName name="_DET_OP_is_between">'_DET Context'!$O$2:$O$5</definedName>
-    <definedName name="_DET_OP_is_email">'_DET Context'!$P$2:$P$2</definedName>
-    <definedName name="_DET_OP_is_in_list">'_DET Context'!$Q$2:$Q$4</definedName>
-    <definedName name="_DET_OP_is_positive">'_DET Context'!$R$2:$R$2</definedName>
-    <definedName name="_DET_OP_lower">'_DET Context'!$S$2:$S$2</definedName>
-    <definedName name="_DET_OP_map_values">'_DET Context'!$T$2:$T$10</definedName>
-    <definedName name="_DET_OP_no_future_date">'_DET Context'!$U$2:$U$2</definedName>
-    <definedName name="_DET_OP_regex_match">'_DET Context'!$V$2:$V$2</definedName>
-    <definedName name="_DET_OP_required">'_DET Context'!$W$2:$W$2</definedName>
-    <definedName name="_DET_OP_rule_compare">'_DET Context'!$X$2:$X$4</definedName>
-    <definedName name="_DET_OP_standardize_country">'_DET Context'!$Y$2:$Y$2</definedName>
-    <definedName name="_DET_OP_standardize_currency">'_DET Context'!$Z$2:$Z$2</definedName>
-    <definedName name="_DET_OP_title">'_DET Context'!$AA$2:$AA$2</definedName>
-    <definedName name="_DET_OP_unique">'_DET Context'!$AB$2:$AB$2</definedName>
-    <definedName name="_DET_OP_upper">'_DET Context'!$AC$2:$AC$2</definedName>
-    <definedName name="_DET_REL_data_product">'_DET Context'!$AD$2:$AD$2</definedName>
-    <definedName name="_DET_VALUE_clean_code_case">'_DET Context'!$AE$2:$AE$4</definedName>
-    <definedName name="_DET_VALUE_clean_text_case">'_DET Context'!$AF$2:$AF$4</definedName>
-    <definedName name="_DET_VALUE_map_values_data_type">'_DET Context'!$AG$2:$AG$7</definedName>
-    <definedName name="_DET_VALUE_map_values_format_case">'_DET Context'!$AH$2:$AH$5</definedName>
-    <definedName name="_DET_VALUE_rule_compare_operator">'_DET Context'!$AI$2:$AI$8</definedName>
+    <definedName name="_DET_OP_convert_value">'_DET Context'!$L$2:$L$4</definedName>
+    <definedName name="_DET_OP_copy">'_DET Context'!$M$2:$M$2</definedName>
+    <definedName name="_DET_OP_correct_errors">'_DET Context'!$N$2:$N$3</definedName>
+    <definedName name="_DET_OP_fill_missing">'_DET Context'!$O$2:$O$2</definedName>
+    <definedName name="_DET_OP_is_between">'_DET Context'!$P$2:$P$5</definedName>
+    <definedName name="_DET_OP_is_email">'_DET Context'!$Q$2:$Q$2</definedName>
+    <definedName name="_DET_OP_is_in_list">'_DET Context'!$R$2:$R$4</definedName>
+    <definedName name="_DET_OP_is_positive">'_DET Context'!$S$2:$S$2</definedName>
+    <definedName name="_DET_OP_lower">'_DET Context'!$T$2:$T$2</definedName>
+    <definedName name="_DET_OP_map_values">'_DET Context'!$U$2:$U$10</definedName>
+    <definedName name="_DET_OP_no_future_date">'_DET Context'!$V$2:$V$2</definedName>
+    <definedName name="_DET_OP_regex_match">'_DET Context'!$W$2:$W$2</definedName>
+    <definedName name="_DET_OP_required">'_DET Context'!$X$2:$X$2</definedName>
+    <definedName name="_DET_OP_rule_compare">'_DET Context'!$Y$2:$Y$4</definedName>
+    <definedName name="_DET_OP_standardize_country">'_DET Context'!$Z$2:$Z$2</definedName>
+    <definedName name="_DET_OP_standardize_currency">'_DET Context'!$AA$2:$AA$2</definedName>
+    <definedName name="_DET_OP_title">'_DET Context'!$AB$2:$AB$2</definedName>
+    <definedName name="_DET_OP_unique">'_DET Context'!$AC$2:$AC$2</definedName>
+    <definedName name="_DET_OP_upper">'_DET Context'!$AD$2:$AD$2</definedName>
+    <definedName name="_DET_REL_data_product">'_DET Context'!$AE$2:$AE$2</definedName>
+    <definedName name="_DET_VALUE_clean_code_case">'_DET Context'!$AF$2:$AF$4</definedName>
+    <definedName name="_DET_VALUE_clean_text_case">'_DET Context'!$AG$2:$AG$4</definedName>
+    <definedName name="_DET_VALUE_convert_value_data_type">'_DET Context'!$AH$2:$AH$7</definedName>
+    <definedName name="_DET_VALUE_map_values_data_type">'_DET Context'!$AI$2:$AI$7</definedName>
+    <definedName name="_DET_VALUE_map_values_format_case">'_DET Context'!$AJ$2:$AJ$5</definedName>
+    <definedName name="_DET_VALUE_rule_compare_operator">'_DET Context'!$AK$2:$AK$8</definedName>
     <definedName name="schema.businessName" localSheetId="2">'Schema stg_customers'!$B$8</definedName>
     <definedName name="schema.dataGranularityDescription" localSheetId="2">'Schema stg_customers'!$B$10</definedName>
     <definedName name="schema.description" localSheetId="2">'Schema stg_customers'!$B$7</definedName>
@@ -928,6 +930,21 @@
 </styleSheet>
 </file>
 
+<file path=xl/comments/comment1.xml><?xml version="1.0" encoding="utf-8"?>
+<comments xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <authors>
+    <author>DET Compiler</author>
+  </authors>
+  <commentList>
+    <comment ref="T13" authorId="0" shapeId="0">
+      <text>
+        <t>Executable before DET Mapping steps. Enter one scalar SQL expression over fields from declared model inputs, for example UPPER(transaction_description). Do not enter SELECT, FROM, WHERE, joins, aliases, or multiple statements. det validate checks syntax using the configured adapter dialect and verifies column references.</t>
+      </text>
+    </comment>
+  </commentList>
+</comments>
+</file>
+
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
 <a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme">
   <a:themeElements>
@@ -1539,7 +1556,7 @@
     <row r="31" ht="16" customHeight="1" s="148">
       <c r="A31" s="44" t="inlineStr">
         <is>
-          <t>dbt_data_engineering_toolkit v2.3.0 workflow</t>
+          <t>dbt_data_engineering_toolkit v4.1.1 workflow</t>
         </is>
       </c>
       <c r="E31" s="13" t="n"/>
@@ -1728,17 +1745,17 @@
       </c>
       <c r="B40" s="51" t="inlineStr">
         <is>
-          <t>Generate, sync, and lint</t>
+          <t>Generate, synchronize, and lint</t>
         </is>
       </c>
       <c r="C40" s="51" t="inlineStr">
         <is>
-          <t>Post-sync ODCS + dbt + SQLFluff</t>
+          <t>dbt package refs use the public toolkit URL by default</t>
         </is>
       </c>
       <c r="D40" s="51" t="inlineStr">
         <is>
-          <t>det generate ...; dbt deps; det check ...</t>
+          <t>det generate ...; det check ...; optionally override DBT_DATA_ENGINEERING_TOOLKIT_GIT_URL for a fork or mirror</t>
         </is>
       </c>
     </row>
@@ -8457,14 +8474,14 @@
     <row r="1" ht="28" customHeight="1" s="148">
       <c r="A1" s="56" t="inlineStr">
         <is>
-          <t>DET Source-to-Target Mapping</t>
+          <t>DET Mapping - ordered transformation pipeline</t>
         </is>
       </c>
     </row>
     <row r="2" ht="32" customHeight="1" s="148">
       <c r="A2" s="60" t="inlineStr">
         <is>
-          <t>Select a model, target, available source field and operation. Put only operation-specific options on DET Parameters.</t>
+          <t>Recommended flow (guidance, not a restriction): scalar ODCS Transform Logic -&gt; convert_value / type-aware clean_* -&gt; standardize_* / correct_errors -&gt; mapping -&gt; fill_missing -&gt; business derivation / target conformance -&gt; validation / routing -&gt; final presentation. Repeat a target field with Step 1, 2, 3... Convert or clean according to target intent; do not clean every source as text. Use mapping format only after semantic and business logic is complete. det validate warns about unusual ordering but permits intentional alternatives.</t>
         </is>
       </c>
     </row>
@@ -9295,8 +9312,8 @@
     <dataValidation sqref="D4:D100" showDropDown="0" showInputMessage="1" showErrorMessage="1" allowBlank="1" errorTitle="Value is out of context" error="Choose a value valid for the selected model, relation, or operation." promptTitle="Context-aware input" prompt="Choose a field from the selected source relation." type="list">
       <formula1>=INDIRECT("_DET_REL_"&amp;SUBSTITUTE(SUBSTITUTE($C4," ","_"),"-","_"))</formula1>
     </dataValidation>
-    <dataValidation sqref="F4:F100" showDropDown="0" showInputMessage="1" showErrorMessage="1" allowBlank="1" errorTitle="Unsupported value" error="Choose a value from the controlled list." promptTitle="Controlled input" prompt="Select a supported value." type="list">
-      <formula1>'_DET Lists'!$A$2:$A$19</formula1>
+    <dataValidation sqref="F4:F100" showDropDown="0" showInputMessage="1" showErrorMessage="1" allowBlank="1" errorTitle="Unsupported value" error="Choose a value from the controlled list." promptTitle="Ordered transformation step" prompt="Choose by intent. Recommended: convert/clean -&gt; standardize/correct -&gt; map -&gt; default -&gt; derive/conform -&gt; validate/route -&gt; present. Alternatives are allowed." type="list">
+      <formula1>'_DET Lists'!$A$2:$A$20</formula1>
     </dataValidation>
   </dataValidations>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -13757,7 +13774,7 @@
     <row r="3" ht="30" customHeight="1" s="148">
       <c r="A3" s="61" t="inlineStr">
         <is>
-          <t>Clean text</t>
+          <t>Convert value</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
@@ -13849,7 +13866,7 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>Clean email</t>
+          <t>Clean text</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
@@ -13936,7 +13953,7 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>Clean phone</t>
+          <t>Clean email</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
@@ -14003,7 +14020,7 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>Clean number</t>
+          <t>Clean phone</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
@@ -14045,7 +14062,7 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>Clean whole number</t>
+          <t>Clean number</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
@@ -14082,7 +14099,7 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>Clean date</t>
+          <t>Clean whole number</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
@@ -14119,7 +14136,7 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>Clean timestamp</t>
+          <t>Clean date</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
@@ -14146,7 +14163,7 @@
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>Clean true/false</t>
+          <t>Clean timestamp</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
@@ -14168,7 +14185,7 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>Clean code</t>
+          <t>Clean true/false</t>
         </is>
       </c>
       <c r="T11" t="inlineStr">
@@ -14180,7 +14197,7 @@
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>Standardise country</t>
+          <t>Clean code</t>
         </is>
       </c>
       <c r="T12" t="inlineStr">
@@ -14192,7 +14209,7 @@
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>Standardise currency</t>
+          <t>Standardise country</t>
         </is>
       </c>
       <c r="T13" t="inlineStr">
@@ -14204,7 +14221,7 @@
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>Map values</t>
+          <t>Standardise currency</t>
         </is>
       </c>
       <c r="T14" t="inlineStr">
@@ -14216,7 +14233,7 @@
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>Fill missing</t>
+          <t>Map values</t>
         </is>
       </c>
       <c r="T15" t="inlineStr">
@@ -14228,7 +14245,7 @@
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>Correct known errors</t>
+          <t>Fill missing</t>
         </is>
       </c>
       <c r="T16" t="inlineStr">
@@ -14240,7 +14257,7 @@
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>Lower case</t>
+          <t>Correct known errors</t>
         </is>
       </c>
       <c r="T17" t="inlineStr">
@@ -14252,7 +14269,7 @@
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>Upper case</t>
+          <t>Lower case</t>
         </is>
       </c>
       <c r="T18" t="inlineStr">
@@ -14264,16 +14281,21 @@
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
+          <t>Upper case</t>
+        </is>
+      </c>
+      <c r="T19" t="inlineStr">
+        <is>
+          <t>Pattern</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
           <t>Title case</t>
         </is>
       </c>
-      <c r="T19" t="inlineStr">
-        <is>
-          <t>Pattern</t>
-        </is>
-      </c>
-    </row>
-    <row r="20">
       <c r="T20" t="inlineStr">
         <is>
           <t>Precision</t>
@@ -14334,7 +14356,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B8"/>
+  <dimension ref="A1:B12"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="30" customWidth="1" style="148" min="1" max="1"/>
@@ -14387,7 +14409,7 @@
       </c>
       <c r="B5" s="152" t="inlineStr">
         <is>
-          <t>2.3.0</t>
+          <t>4.1.1</t>
         </is>
       </c>
     </row>
@@ -14399,7 +14421,7 @@
       </c>
       <c r="B6" s="152" t="inlineStr">
         <is>
-          <t>2.3.0</t>
+          <t>4.1.1</t>
         </is>
       </c>
     </row>
@@ -14411,7 +14433,7 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>1429ce4f80e5f9adf552a3fd404d94b7e7a0cd98434fff6fafe63717a8a6b8cf</t>
+          <t>9cf184d87d656fdec8fe3ae1bcf6d1d769f84995baf0fcc1ee89b6ede9e5277f</t>
         </is>
       </c>
     </row>
@@ -14427,6 +14449,10 @@
         </is>
       </c>
     </row>
+    <row r="9"/>
+    <row r="10"/>
+    <row r="11"/>
+    <row r="12"/>
   </sheetData>
   <sheetProtection selectLockedCells="0" selectUnlockedCells="0" sheet="1" objects="0" insertRows="1" insertHyperlinks="1" autoFilter="1" scenarios="0" formatColumns="1" deleteColumns="1" insertColumns="1" pivotTables="1" deleteRows="1" formatCells="1" formatRows="1" sort="1" password="CCB4"/>
   <mergeCells count="2">
@@ -14443,7 +14469,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AI10"/>
+  <dimension ref="A1:AK10"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -14504,131 +14530,147 @@
       </c>
       <c r="L1" t="inlineStr">
         <is>
+          <t>_DET_OP_convert_value</t>
+        </is>
+      </c>
+      <c r="M1" t="inlineStr">
+        <is>
           <t>_DET_OP_copy</t>
         </is>
       </c>
-      <c r="M1" t="inlineStr">
+      <c r="N1" t="inlineStr">
         <is>
           <t>_DET_OP_correct_errors</t>
         </is>
       </c>
-      <c r="N1" t="inlineStr">
+      <c r="O1" t="inlineStr">
         <is>
           <t>_DET_OP_fill_missing</t>
         </is>
       </c>
-      <c r="O1" t="inlineStr">
+      <c r="P1" t="inlineStr">
         <is>
           <t>_DET_OP_is_between</t>
         </is>
       </c>
-      <c r="P1" t="inlineStr">
+      <c r="Q1" t="inlineStr">
         <is>
           <t>_DET_OP_is_email</t>
         </is>
       </c>
-      <c r="Q1" t="inlineStr">
+      <c r="R1" t="inlineStr">
         <is>
           <t>_DET_OP_is_in_list</t>
         </is>
       </c>
-      <c r="R1" t="inlineStr">
+      <c r="S1" t="inlineStr">
         <is>
           <t>_DET_OP_is_positive</t>
         </is>
       </c>
-      <c r="S1" t="inlineStr">
+      <c r="T1" t="inlineStr">
         <is>
           <t>_DET_OP_lower</t>
         </is>
       </c>
-      <c r="T1" t="inlineStr">
+      <c r="U1" t="inlineStr">
         <is>
           <t>_DET_OP_map_values</t>
         </is>
       </c>
-      <c r="U1" t="inlineStr">
+      <c r="V1" t="inlineStr">
         <is>
           <t>_DET_OP_no_future_date</t>
         </is>
       </c>
-      <c r="V1" t="inlineStr">
+      <c r="W1" t="inlineStr">
         <is>
           <t>_DET_OP_regex_match</t>
         </is>
       </c>
-      <c r="W1" t="inlineStr">
+      <c r="X1" t="inlineStr">
         <is>
           <t>_DET_OP_required</t>
         </is>
       </c>
-      <c r="X1" t="inlineStr">
+      <c r="Y1" t="inlineStr">
         <is>
           <t>_DET_OP_rule_compare</t>
         </is>
       </c>
-      <c r="Y1" t="inlineStr">
+      <c r="Z1" t="inlineStr">
         <is>
           <t>_DET_OP_standardize_country</t>
         </is>
       </c>
-      <c r="Z1" t="inlineStr">
+      <c r="AA1" t="inlineStr">
         <is>
           <t>_DET_OP_standardize_currency</t>
         </is>
       </c>
-      <c r="AA1" t="inlineStr">
+      <c r="AB1" t="inlineStr">
         <is>
           <t>_DET_OP_title</t>
         </is>
       </c>
-      <c r="AB1" t="inlineStr">
+      <c r="AC1" t="inlineStr">
         <is>
           <t>_DET_OP_unique</t>
         </is>
       </c>
-      <c r="AC1" t="inlineStr">
+      <c r="AD1" t="inlineStr">
         <is>
           <t>_DET_OP_upper</t>
         </is>
       </c>
-      <c r="AD1" t="inlineStr">
+      <c r="AE1" t="inlineStr">
         <is>
           <t>_DET_REL_data_product</t>
         </is>
       </c>
-      <c r="AE1" t="inlineStr">
+      <c r="AF1" t="inlineStr">
         <is>
           <t>_DET_VALUE_clean_code_case</t>
         </is>
       </c>
-      <c r="AF1" t="inlineStr">
+      <c r="AG1" t="inlineStr">
         <is>
           <t>_DET_VALUE_clean_text_case</t>
         </is>
       </c>
-      <c r="AG1" t="inlineStr">
+      <c r="AH1" t="inlineStr">
+        <is>
+          <t>_DET_VALUE_convert_value_data_type</t>
+        </is>
+      </c>
+      <c r="AI1" t="inlineStr">
         <is>
           <t>_DET_VALUE_map_values_data_type</t>
         </is>
       </c>
-      <c r="AH1" t="inlineStr">
+      <c r="AJ1" t="inlineStr">
         <is>
           <t>_DET_VALUE_map_values_format_case</t>
         </is>
       </c>
-      <c r="AI1" t="inlineStr">
+      <c r="AK1" t="inlineStr">
         <is>
           <t>_DET_VALUE_rule_compare_operator</t>
         </is>
       </c>
     </row>
     <row r="2">
+      <c r="A2" t="inlineStr"/>
+      <c r="B2" t="inlineStr"/>
+      <c r="C2" t="inlineStr"/>
       <c r="D2" t="inlineStr">
         <is>
           <t>Remove Prefix</t>
         </is>
       </c>
+      <c r="E2" t="inlineStr"/>
+      <c r="F2" t="inlineStr"/>
+      <c r="G2" t="inlineStr"/>
       <c r="H2" t="inlineStr">
         <is>
           <t>Precision</t>
@@ -14644,72 +14686,93 @@
           <t>Trim</t>
         </is>
       </c>
-      <c r="M2" t="inlineStr">
+      <c r="K2" t="inlineStr"/>
+      <c r="L2" t="inlineStr">
+        <is>
+          <t>Data Type</t>
+        </is>
+      </c>
+      <c r="M2" t="inlineStr"/>
+      <c r="N2" t="inlineStr">
         <is>
           <t>Lookup</t>
         </is>
       </c>
-      <c r="N2" t="inlineStr">
+      <c r="O2" t="inlineStr">
         <is>
           <t>Fill Value</t>
         </is>
       </c>
-      <c r="O2" t="inlineStr">
+      <c r="P2" t="inlineStr">
         <is>
           <t>Minimum</t>
         </is>
       </c>
-      <c r="P2" t="inlineStr">
+      <c r="Q2" t="inlineStr">
         <is>
           <t>Allow Null</t>
         </is>
       </c>
-      <c r="Q2" t="inlineStr">
+      <c r="R2" t="inlineStr">
         <is>
           <t>Values</t>
         </is>
       </c>
-      <c r="R2" t="inlineStr">
+      <c r="S2" t="inlineStr">
         <is>
           <t>Allow Null</t>
         </is>
       </c>
-      <c r="T2" t="inlineStr">
+      <c r="T2" t="inlineStr"/>
+      <c r="U2" t="inlineStr">
         <is>
           <t>Lookup</t>
         </is>
       </c>
-      <c r="V2" t="inlineStr">
+      <c r="V2" t="inlineStr"/>
+      <c r="W2" t="inlineStr">
         <is>
           <t>Pattern</t>
         </is>
       </c>
-      <c r="X2" t="inlineStr">
+      <c r="X2" t="inlineStr"/>
+      <c r="Y2" t="inlineStr">
         <is>
           <t>Operator</t>
         </is>
       </c>
-      <c r="AE2" t="inlineStr">
+      <c r="Z2" t="inlineStr"/>
+      <c r="AA2" t="inlineStr"/>
+      <c r="AB2" t="inlineStr"/>
+      <c r="AC2" t="inlineStr"/>
+      <c r="AD2" t="inlineStr"/>
+      <c r="AE2" t="inlineStr"/>
+      <c r="AF2" t="inlineStr">
         <is>
           <t>preserve</t>
         </is>
       </c>
-      <c r="AF2" t="inlineStr">
+      <c r="AG2" t="inlineStr">
         <is>
           <t>preserve</t>
         </is>
       </c>
-      <c r="AG2" t="inlineStr">
+      <c r="AH2" t="inlineStr">
         <is>
           <t>string</t>
         </is>
       </c>
-      <c r="AH2" t="inlineStr">
+      <c r="AI2" t="inlineStr">
+        <is>
+          <t>string</t>
+        </is>
+      </c>
+      <c r="AJ2" t="inlineStr">
         <is>
           <t>preserve</t>
         </is>
       </c>
-      <c r="AI2" t="inlineStr">
+      <c r="AK2" t="inlineStr">
         <is>
           <t>=</t>
         </is>
@@ -14731,52 +14794,62 @@
           <t>Collapse Whitespace</t>
         </is>
       </c>
-      <c r="M3" t="inlineStr">
+      <c r="L3" t="inlineStr">
+        <is>
+          <t>Precision</t>
+        </is>
+      </c>
+      <c r="N3" t="inlineStr">
         <is>
           <t>Case Sensitive</t>
         </is>
       </c>
-      <c r="O3" t="inlineStr">
+      <c r="P3" t="inlineStr">
         <is>
           <t>Maximum</t>
         </is>
       </c>
-      <c r="Q3" t="inlineStr">
+      <c r="R3" t="inlineStr">
         <is>
           <t>Allow Null</t>
         </is>
       </c>
-      <c r="T3" t="inlineStr">
+      <c r="U3" t="inlineStr">
         <is>
           <t>Default</t>
         </is>
       </c>
-      <c r="X3" t="inlineStr">
+      <c r="Y3" t="inlineStr">
         <is>
           <t>Compare To</t>
         </is>
       </c>
-      <c r="AE3" t="inlineStr">
+      <c r="AF3" t="inlineStr">
         <is>
           <t>lower</t>
         </is>
       </c>
-      <c r="AF3" t="inlineStr">
+      <c r="AG3" t="inlineStr">
         <is>
           <t>lower</t>
         </is>
       </c>
-      <c r="AG3" t="inlineStr">
+      <c r="AH3" t="inlineStr">
         <is>
           <t>integer</t>
         </is>
       </c>
-      <c r="AH3" t="inlineStr">
+      <c r="AI3" t="inlineStr">
+        <is>
+          <t>integer</t>
+        </is>
+      </c>
+      <c r="AJ3" t="inlineStr">
         <is>
           <t>lower</t>
         </is>
       </c>
-      <c r="AI3" t="inlineStr">
+      <c r="AK3" t="inlineStr">
         <is>
           <t>!=</t>
         </is>
@@ -14793,47 +14866,57 @@
           <t>Case</t>
         </is>
       </c>
-      <c r="O4" t="inlineStr">
+      <c r="L4" t="inlineStr">
+        <is>
+          <t>Scale</t>
+        </is>
+      </c>
+      <c r="P4" t="inlineStr">
         <is>
           <t>Inclusive</t>
         </is>
       </c>
-      <c r="Q4" t="inlineStr">
+      <c r="R4" t="inlineStr">
         <is>
           <t>Case Sensitive</t>
         </is>
       </c>
-      <c r="T4" t="inlineStr">
+      <c r="U4" t="inlineStr">
         <is>
           <t>Preserve Unmapped</t>
         </is>
       </c>
-      <c r="X4" t="inlineStr">
+      <c r="Y4" t="inlineStr">
         <is>
           <t>Allow Null</t>
         </is>
       </c>
-      <c r="AE4" t="inlineStr">
+      <c r="AF4" t="inlineStr">
         <is>
           <t>upper</t>
         </is>
       </c>
-      <c r="AF4" t="inlineStr">
+      <c r="AG4" t="inlineStr">
         <is>
           <t>upper</t>
         </is>
       </c>
-      <c r="AG4" t="inlineStr">
+      <c r="AH4" t="inlineStr">
         <is>
           <t>numeric</t>
         </is>
       </c>
-      <c r="AH4" t="inlineStr">
+      <c r="AI4" t="inlineStr">
+        <is>
+          <t>numeric</t>
+        </is>
+      </c>
+      <c r="AJ4" t="inlineStr">
         <is>
           <t>upper</t>
         </is>
       </c>
-      <c r="AI4" t="inlineStr">
+      <c r="AK4" t="inlineStr">
         <is>
           <t>&lt;&gt;</t>
         </is>
@@ -14850,87 +14933,102 @@
           <t>Blank As Null</t>
         </is>
       </c>
-      <c r="O5" t="inlineStr">
+      <c r="P5" t="inlineStr">
         <is>
           <t>Allow Null</t>
         </is>
       </c>
-      <c r="T5" t="inlineStr">
+      <c r="U5" t="inlineStr">
         <is>
           <t>Case Sensitive</t>
         </is>
       </c>
-      <c r="AG5" t="inlineStr">
+      <c r="AH5" t="inlineStr">
         <is>
           <t>date</t>
         </is>
       </c>
-      <c r="AH5" t="inlineStr">
+      <c r="AI5" t="inlineStr">
+        <is>
+          <t>date</t>
+        </is>
+      </c>
+      <c r="AJ5" t="inlineStr">
         <is>
           <t>title</t>
         </is>
       </c>
-      <c r="AI5" t="inlineStr">
+      <c r="AK5" t="inlineStr">
         <is>
           <t>&lt;</t>
         </is>
       </c>
     </row>
     <row r="6">
-      <c r="T6" t="inlineStr">
+      <c r="U6" t="inlineStr">
         <is>
           <t>Data Type</t>
         </is>
       </c>
-      <c r="AG6" t="inlineStr">
+      <c r="AH6" t="inlineStr">
         <is>
           <t>timestamp</t>
         </is>
       </c>
       <c r="AI6" t="inlineStr">
         <is>
+          <t>timestamp</t>
+        </is>
+      </c>
+      <c r="AK6" t="inlineStr">
+        <is>
           <t>&lt;=</t>
         </is>
       </c>
     </row>
     <row r="7">
-      <c r="T7" t="inlineStr">
+      <c r="U7" t="inlineStr">
         <is>
           <t>Precision</t>
         </is>
       </c>
-      <c r="AG7" t="inlineStr">
+      <c r="AH7" t="inlineStr">
         <is>
           <t>boolean</t>
         </is>
       </c>
       <c r="AI7" t="inlineStr">
         <is>
+          <t>boolean</t>
+        </is>
+      </c>
+      <c r="AK7" t="inlineStr">
+        <is>
           <t>&gt;</t>
         </is>
       </c>
     </row>
     <row r="8">
-      <c r="T8" t="inlineStr">
+      <c r="U8" t="inlineStr">
         <is>
           <t>Scale</t>
         </is>
       </c>
-      <c r="AI8" t="inlineStr">
+      <c r="AK8" t="inlineStr">
         <is>
           <t>&gt;=</t>
         </is>
       </c>
     </row>
     <row r="9">
-      <c r="T9" t="inlineStr">
+      <c r="U9" t="inlineStr">
         <is>
           <t>Format Pattern</t>
         </is>
       </c>
     </row>
     <row r="10">
-      <c r="T10" t="inlineStr">
+      <c r="U10" t="inlineStr">
         <is>
           <t>Format Case</t>
         </is>
@@ -14992,8 +15090,8 @@
     <col hidden="1" outlineLevel="1" width="13" customWidth="1" style="148" min="17" max="17"/>
     <col hidden="1" outlineLevel="1" width="13" customWidth="1" style="148" min="18" max="18"/>
     <col hidden="1" outlineLevel="1" width="13" customWidth="1" style="148" min="19" max="19"/>
-    <col hidden="1" outlineLevel="1" width="13" customWidth="1" style="148" min="20" max="20"/>
-    <col hidden="1" outlineLevel="1" width="21.6640625" customWidth="1" style="2" min="21" max="21"/>
+    <col width="42" customWidth="1" style="148" min="20" max="20"/>
+    <col width="32" customWidth="1" style="2" min="21" max="21"/>
     <col hidden="1" outlineLevel="1" width="27.33203125" customWidth="1" style="2" min="22" max="22"/>
     <col hidden="1" outlineLevel="1" width="15.5" customWidth="1" style="2" min="23" max="37"/>
     <col hidden="1" outlineLevel="1" width="13" customWidth="1" style="148" min="24" max="24"/>
@@ -18916,7 +19014,16 @@
     <mergeCell ref="B5:E5"/>
     <mergeCell ref="B10:E10"/>
   </mergeCells>
-  <dataValidations count="15">
+  <dataValidations count="18">
+    <dataValidation sqref="AM14:AM100" showDropDown="0" showInputMessage="1" showErrorMessage="1" allowBlank="1" errorTitle="Unsupported value" error="Choose a value from the controlled list." promptTitle="Controlled input" prompt="Select a supported value." type="list">
+      <formula1>'_DET Lists'!$U$2:$U$4</formula1>
+    </dataValidation>
+    <dataValidation sqref="AM14:AM100" showDropDown="0" showInputMessage="1" showErrorMessage="1" allowBlank="1" errorTitle="Unsupported value" error="Choose a value from the controlled list." promptTitle="Controlled input" prompt="Select a supported value." type="list">
+      <formula1>'_DET Lists'!$U$2:$U$4</formula1>
+    </dataValidation>
+    <dataValidation sqref="AM14:AM100" showDropDown="0" showInputMessage="1" showErrorMessage="1" allowBlank="1" errorTitle="Unsupported value" error="Choose a value from the controlled list." promptTitle="Controlled input" prompt="Select a supported value." type="list">
+      <formula1>'_DET Lists'!$U$2:$U$4</formula1>
+    </dataValidation>
     <dataValidation sqref="AM14:AM100" showDropDown="0" showInputMessage="1" showErrorMessage="1" allowBlank="1" errorTitle="Unsupported value" error="Choose a value from the controlled list." promptTitle="Controlled input" prompt="Select a supported value." type="list">
       <formula1>'_DET Lists'!$U$2:$U$4</formula1>
     </dataValidation>
@@ -18964,6 +19071,7 @@
     </dataValidation>
   </dataValidations>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <legacyDrawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="anysvml"/>
 </worksheet>
 </file>
 

</xml_diff>

<commit_message>
update versioning to be semantic without the preceding 'v'
</commit_message>
<xml_diff>
--- a/python/src/dbt_data_engineering_toolkit_compiler/resources/data_product.xlsx
+++ b/python/src/dbt_data_engineering_toolkit_compiler/resources/data_product.xlsx
@@ -13461,7 +13461,7 @@
       </c>
       <c r="B8" s="166" t="inlineStr">
         <is>
-          <t>v4.1.1</t>
+          <t>4.1.1</t>
         </is>
       </c>
       <c r="C8" s="152" t="inlineStr">
@@ -14356,7 +14356,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B12"/>
+  <dimension ref="A1:B8"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="30" customWidth="1" style="148" min="1" max="1"/>
@@ -14449,10 +14449,6 @@
         </is>
       </c>
     </row>
-    <row r="9"/>
-    <row r="10"/>
-    <row r="11"/>
-    <row r="12"/>
   </sheetData>
   <sheetProtection selectLockedCells="0" selectUnlockedCells="0" sheet="1" objects="0" insertRows="1" insertHyperlinks="1" autoFilter="1" scenarios="0" formatColumns="1" deleteColumns="1" insertColumns="1" pivotTables="1" deleteRows="1" formatCells="1" formatRows="1" sort="1" password="CCB4"/>
   <mergeCells count="2">
@@ -14660,17 +14656,11 @@
       </c>
     </row>
     <row r="2">
-      <c r="A2" t="inlineStr"/>
-      <c r="B2" t="inlineStr"/>
-      <c r="C2" t="inlineStr"/>
       <c r="D2" t="inlineStr">
         <is>
           <t>Remove Prefix</t>
         </is>
       </c>
-      <c r="E2" t="inlineStr"/>
-      <c r="F2" t="inlineStr"/>
-      <c r="G2" t="inlineStr"/>
       <c r="H2" t="inlineStr">
         <is>
           <t>Precision</t>
@@ -14686,13 +14676,11 @@
           <t>Trim</t>
         </is>
       </c>
-      <c r="K2" t="inlineStr"/>
       <c r="L2" t="inlineStr">
         <is>
           <t>Data Type</t>
         </is>
       </c>
-      <c r="M2" t="inlineStr"/>
       <c r="N2" t="inlineStr">
         <is>
           <t>Lookup</t>
@@ -14723,30 +14711,21 @@
           <t>Allow Null</t>
         </is>
       </c>
-      <c r="T2" t="inlineStr"/>
       <c r="U2" t="inlineStr">
         <is>
           <t>Lookup</t>
         </is>
       </c>
-      <c r="V2" t="inlineStr"/>
       <c r="W2" t="inlineStr">
         <is>
           <t>Pattern</t>
         </is>
       </c>
-      <c r="X2" t="inlineStr"/>
       <c r="Y2" t="inlineStr">
         <is>
           <t>Operator</t>
         </is>
       </c>
-      <c r="Z2" t="inlineStr"/>
-      <c r="AA2" t="inlineStr"/>
-      <c r="AB2" t="inlineStr"/>
-      <c r="AC2" t="inlineStr"/>
-      <c r="AD2" t="inlineStr"/>
-      <c r="AE2" t="inlineStr"/>
       <c r="AF2" t="inlineStr">
         <is>
           <t>preserve</t>

</xml_diff>

<commit_message>
bump version 4.1.1 -> 5.0.0
</commit_message>
<xml_diff>
--- a/python/src/dbt_data_engineering_toolkit_compiler/resources/data_product.xlsx
+++ b/python/src/dbt_data_engineering_toolkit_compiler/resources/data_product.xlsx
@@ -1,35 +1,35 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Instructions" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Fundamentals" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Schema data_product" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Relationships" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Quality" sheetId="5" state="visible" r:id="rId5"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Support" sheetId="6" state="visible" r:id="rId6"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Team" sheetId="7" state="visible" r:id="rId7"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Roles" sheetId="8" state="visible" r:id="rId8"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SLA" sheetId="9" state="visible" r:id="rId9"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Servers" sheetId="10" state="visible" r:id="rId10"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Pricing" sheetId="11" state="visible" r:id="rId11"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Custom Properties" sheetId="12" state="visible" r:id="rId12"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="DET Models" sheetId="13" state="visible" r:id="rId13"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="DET Model Inputs" sheetId="14" state="visible" r:id="rId14"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="DET Sources" sheetId="15" state="visible" r:id="rId15"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="DET Source Schema" sheetId="16" state="visible" r:id="rId16"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="DET Mapping" sheetId="17" state="visible" r:id="rId17"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="DET Parameters" sheetId="18" state="visible" r:id="rId18"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="DET Relationships" sheetId="19" state="visible" r:id="rId19"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Operational Validation" sheetId="20" state="visible" r:id="rId20"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Operational Parameters" sheetId="21" state="visible" r:id="rId21"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="DET Lookups" sheetId="22" state="visible" r:id="rId22"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="DET Build" sheetId="23" state="visible" r:id="rId23"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="_DET Lists" sheetId="24" state="veryHidden" r:id="rId24"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="_DET Metadata" sheetId="25" state="veryHidden" r:id="rId25"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="_DET Context" sheetId="26" state="veryHidden" r:id="rId26"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="_DET Raw ODCS" sheetId="27" state="veryHidden" r:id="rId27"/>
+    <sheet name="Instructions" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Fundamentals" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="Schema data_product" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="Relationships" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet name="Quality" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet name="Support" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet name="Team" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet name="Roles" sheetId="8" state="visible" r:id="rId8"/>
+    <sheet name="SLA" sheetId="9" state="visible" r:id="rId9"/>
+    <sheet name="Servers" sheetId="10" state="visible" r:id="rId10"/>
+    <sheet name="Pricing" sheetId="11" state="visible" r:id="rId11"/>
+    <sheet name="Custom Properties" sheetId="12" state="visible" r:id="rId12"/>
+    <sheet name="DET Models" sheetId="13" state="visible" r:id="rId13"/>
+    <sheet name="DET Model Inputs" sheetId="14" state="visible" r:id="rId14"/>
+    <sheet name="DET Sources" sheetId="15" state="visible" r:id="rId15"/>
+    <sheet name="DET Source Schema" sheetId="16" state="visible" r:id="rId16"/>
+    <sheet name="DET Mapping" sheetId="17" state="visible" r:id="rId17"/>
+    <sheet name="DET Parameters" sheetId="18" state="visible" r:id="rId18"/>
+    <sheet name="DET Relationships" sheetId="19" state="visible" r:id="rId19"/>
+    <sheet name="Operational Validation" sheetId="20" state="visible" r:id="rId20"/>
+    <sheet name="Operational Parameters" sheetId="21" state="visible" r:id="rId21"/>
+    <sheet name="DET Lookups" sheetId="22" state="visible" r:id="rId22"/>
+    <sheet name="DET Build" sheetId="23" state="visible" r:id="rId23"/>
+    <sheet name="_DET Lists" sheetId="24" state="veryHidden" r:id="rId24"/>
+    <sheet name="_DET Metadata" sheetId="25" state="veryHidden" r:id="rId25"/>
+    <sheet name="_DET Context" sheetId="26" state="veryHidden" r:id="rId26"/>
+    <sheet name="_DET Raw ODCS" sheetId="27" state="veryHidden" r:id="rId27"/>
   </sheets>
   <definedNames>
     <definedName name="apiVersion">Fundamentals!$C$5</definedName>
@@ -13461,7 +13461,7 @@
       </c>
       <c r="B8" s="166" t="inlineStr">
         <is>
-          <t>4.1.1</t>
+          <t>5.0.0</t>
         </is>
       </c>
       <c r="C8" s="152" t="inlineStr">
@@ -14397,7 +14397,7 @@
       </c>
       <c r="B4" s="152" t="inlineStr">
         <is>
-          <t>4.1.1</t>
+          <t>5.0.0</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
bump version 5.0.0 -> 5.0.1
</commit_message>
<xml_diff>
--- a/python/src/dbt_data_engineering_toolkit_compiler/resources/data_product.xlsx
+++ b/python/src/dbt_data_engineering_toolkit_compiler/resources/data_product.xlsx
@@ -13461,7 +13461,7 @@
       </c>
       <c r="B8" s="166" t="inlineStr">
         <is>
-          <t>5.0.0</t>
+          <t>5.0.1</t>
         </is>
       </c>
       <c r="C8" s="152" t="inlineStr">
@@ -14397,7 +14397,7 @@
       </c>
       <c r="B4" s="152" t="inlineStr">
         <is>
-          <t>5.0.0</t>
+          <t>5.0.1</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
bump version 5.0.1 -> 6.0.0
</commit_message>
<xml_diff>
--- a/python/src/dbt_data_engineering_toolkit_compiler/resources/data_product.xlsx
+++ b/python/src/dbt_data_engineering_toolkit_compiler/resources/data_product.xlsx
@@ -13461,7 +13461,7 @@
       </c>
       <c r="B8" s="166" t="inlineStr">
         <is>
-          <t>5.0.1</t>
+          <t>6.0.0</t>
         </is>
       </c>
       <c r="C8" s="152" t="inlineStr">
@@ -14397,7 +14397,7 @@
       </c>
       <c r="B4" s="152" t="inlineStr">
         <is>
-          <t>5.0.1</t>
+          <t>6.0.0</t>
         </is>
       </c>
     </row>

</xml_diff>